<commit_message>
workflow(variation): complete publication artifacts
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -3643,7 +3643,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>checked</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3663,17 +3663,17 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>review evidence invalidated; original body and raw records preserved; independent review and known content corrections remain pending</t>
+          <t>source-first inventory; seven independent checker passes and affected-pass rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">

</xml_diff>

<commit_message>
entry(definite): publish checked dictionary entry
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3729,6 +3729,58 @@
         </is>
       </c>
       <c r="J64" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>definite</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E65" s="1" t="inlineStr">
+        <is>
+          <t>entries/d/definite.md</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven checker passes with affected-pass rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3799,6 +3851,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
entry(definite): add checked dictionary entry (#173)
Add the v5 definite entry with source-first audit, reviews, and exports.
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3729,6 +3729,58 @@
         </is>
       </c>
       <c r="J64" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>definite</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E65" s="1" t="inlineStr">
+        <is>
+          <t>entries/d/definite.md</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven checker passes with affected-pass rechecks; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3799,6 +3851,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
workflow(tentative): finalize checked entry
</commit_message>
<xml_diff>
--- a/exports/dictionary_index.xlsx
+++ b/exports/dictionary_index.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3781,6 +3781,110 @@
         </is>
       </c>
       <c r="J65" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>appropriate</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="E66" s="1" t="inlineStr">
+        <is>
+          <t>entries/a/appropriate.md</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven checker passes with preserved handoff provenance; context-free cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>word</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>checked</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E67" s="1" t="inlineStr">
+        <is>
+          <t>entries/t/tentative.md</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>entry_spec_v5</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>source-first inventory; seven checker passes and affected-pass recheck; cold review; sealed final blind review; final reconciliation passed</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3852,6 +3956,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId66"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>